<commit_message>
Ship v5.4.2 with progression data, combat depth, and UI consolidation.
Restore spreadsheet-backed stat gains, XP curve, and monster levels so level-ups and regional mob gating work correctly. Add ambush rolls, INT-scaled spells, randomized preset parties, ruins minimap placeholder, and nest Quest/Party and In Memoriam/Church tabs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/chart for game.xlsx
+++ b/chart for game.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/los/Illirial-Trail/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94C0760-1760-7548-88A4-B4AC5FA46482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE4A404A-AC48-A942-A47A-145020AEDF87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1460" yWindow="1400" windowWidth="27660" windowHeight="16680" activeTab="5" xr2:uid="{F86F549B-5A31-4F42-A680-6D6C856460C8}"/>
+    <workbookView xWindow="1460" yWindow="1400" windowWidth="27660" windowHeight="16680" activeTab="6" xr2:uid="{F86F549B-5A31-4F42-A680-6D6C856460C8}"/>
   </bookViews>
   <sheets>
     <sheet name="weapons" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="level testing" sheetId="4" r:id="rId4"/>
     <sheet name="alpha level to 20" sheetId="5" r:id="rId5"/>
     <sheet name="Stat gains per class" sheetId="6" r:id="rId6"/>
+    <sheet name="Names" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="310">
   <si>
     <t>Weapons</t>
   </si>
@@ -659,13 +660,328 @@
   </si>
   <si>
     <t>1 luck = .01% crit. Crit is 200% damage.</t>
+  </si>
+  <si>
+    <t>Names</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Mateus</t>
+  </si>
+  <si>
+    <t>Aramar</t>
+  </si>
+  <si>
+    <t>Aendather</t>
+  </si>
+  <si>
+    <t>Ben</t>
+  </si>
+  <si>
+    <t>Ander</t>
+  </si>
+  <si>
+    <t>Alexander</t>
+  </si>
+  <si>
+    <t>Grace</t>
+  </si>
+  <si>
+    <t>Evelyn</t>
+  </si>
+  <si>
+    <t>Allura</t>
+  </si>
+  <si>
+    <t>Amanda</t>
+  </si>
+  <si>
+    <t>Aurelia</t>
+  </si>
+  <si>
+    <t>Amelia</t>
+  </si>
+  <si>
+    <t>Emileigh</t>
+  </si>
+  <si>
+    <t>Alyene</t>
+  </si>
+  <si>
+    <t>Anderson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anders </t>
+  </si>
+  <si>
+    <t>Beth</t>
+  </si>
+  <si>
+    <t>Belynda</t>
+  </si>
+  <si>
+    <t>Bianca</t>
+  </si>
+  <si>
+    <t>Catherine</t>
+  </si>
+  <si>
+    <t>Carla</t>
+  </si>
+  <si>
+    <t>Elizabeth</t>
+  </si>
+  <si>
+    <t>Elisha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eliza </t>
+  </si>
+  <si>
+    <t>Eris</t>
+  </si>
+  <si>
+    <t>Aerie</t>
+  </si>
+  <si>
+    <t>Zelda</t>
+  </si>
+  <si>
+    <t>Fiona</t>
+  </si>
+  <si>
+    <t>Ryona</t>
+  </si>
+  <si>
+    <t>Helene</t>
+  </si>
+  <si>
+    <t>Helena</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Jacqueline</t>
+  </si>
+  <si>
+    <t>Brian</t>
+  </si>
+  <si>
+    <t>Bryan</t>
+  </si>
+  <si>
+    <t>Brandon</t>
+  </si>
+  <si>
+    <t>Brayden</t>
+  </si>
+  <si>
+    <t>Brocca</t>
+  </si>
+  <si>
+    <t>Benjamin</t>
+  </si>
+  <si>
+    <t>Benni</t>
+  </si>
+  <si>
+    <t>Chalice</t>
+  </si>
+  <si>
+    <t>Desinty</t>
+  </si>
+  <si>
+    <t>Desmond</t>
+  </si>
+  <si>
+    <t>Derrick</t>
+  </si>
+  <si>
+    <t>Deryk</t>
+  </si>
+  <si>
+    <t>Dionysus</t>
+  </si>
+  <si>
+    <t>Erik</t>
+  </si>
+  <si>
+    <t>Eric</t>
+  </si>
+  <si>
+    <t>Erica</t>
+  </si>
+  <si>
+    <t>Jessica</t>
+  </si>
+  <si>
+    <t>Jessie</t>
+  </si>
+  <si>
+    <t>Jeryca</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Jon</t>
+  </si>
+  <si>
+    <t>Jonathan</t>
+  </si>
+  <si>
+    <t>Jonathon</t>
+  </si>
+  <si>
+    <t>Jeremiah</t>
+  </si>
+  <si>
+    <t>Jericho</t>
+  </si>
+  <si>
+    <t>Lamont</t>
+  </si>
+  <si>
+    <t>Layton</t>
+  </si>
+  <si>
+    <t>Luke</t>
+  </si>
+  <si>
+    <t>Liam</t>
+  </si>
+  <si>
+    <t>Kimberly</t>
+  </si>
+  <si>
+    <t>Kathryn</t>
+  </si>
+  <si>
+    <t>Lisa</t>
+  </si>
+  <si>
+    <t>Liz</t>
+  </si>
+  <si>
+    <t>Martha</t>
+  </si>
+  <si>
+    <t>Mary</t>
+  </si>
+  <si>
+    <t>Mandy</t>
+  </si>
+  <si>
+    <t>Nicole</t>
+  </si>
+  <si>
+    <t>Nicola</t>
+  </si>
+  <si>
+    <t>Michelle</t>
+  </si>
+  <si>
+    <t>Michael</t>
+  </si>
+  <si>
+    <t>Mick</t>
+  </si>
+  <si>
+    <t>Michel</t>
+  </si>
+  <si>
+    <t>Hikaru</t>
+  </si>
+  <si>
+    <t>Isamu</t>
+  </si>
+  <si>
+    <t>Hibiki</t>
+  </si>
+  <si>
+    <t>Nichelle</t>
+  </si>
+  <si>
+    <t>Ophilia</t>
+  </si>
+  <si>
+    <t>Pamela</t>
+  </si>
+  <si>
+    <t>Rosa</t>
+  </si>
+  <si>
+    <t>Rosalinda</t>
+  </si>
+  <si>
+    <t>Rachel</t>
+  </si>
+  <si>
+    <t>Rachelle</t>
+  </si>
+  <si>
+    <t>Samantha</t>
+  </si>
+  <si>
+    <t>Sandra</t>
+  </si>
+  <si>
+    <t>Sadie</t>
+  </si>
+  <si>
+    <t>Terri</t>
+  </si>
+  <si>
+    <t>Uelda</t>
+  </si>
+  <si>
+    <t>Viera</t>
+  </si>
+  <si>
+    <t>Ilsa</t>
+  </si>
+  <si>
+    <t>Iliana</t>
+  </si>
+  <si>
+    <t>Jean</t>
+  </si>
+  <si>
+    <t>William</t>
+  </si>
+  <si>
+    <t>Jeordy</t>
+  </si>
+  <si>
+    <t>Austin</t>
+  </si>
+  <si>
+    <t>Bradley</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brad </t>
+  </si>
+  <si>
+    <t>James</t>
+  </si>
+  <si>
+    <t>Jamison</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -697,6 +1013,13 @@
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="24"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -847,7 +1170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -874,18 +1197,6 @@
     <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -900,13 +1211,29 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4819,17 +5146,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B2" s="16" t="s">
@@ -5010,10 +5337,10 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="34" t="s">
         <v>152</v>
       </c>
-      <c r="C8" s="22"/>
+      <c r="C8" s="35"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C9" s="18">
@@ -5207,14 +5534,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27" x14ac:dyDescent="0.35">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="36" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -5845,7 +6172,7 @@
         <v>4</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C22" si="0">B5-B4</f>
+        <f t="shared" ref="C4:C21" si="0">B5-B4</f>
         <v>2</v>
       </c>
     </row>
@@ -6076,285 +6403,285 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="24"/>
-      <c r="B1" s="25" t="s">
+      <c r="A1" s="20"/>
+      <c r="B1" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="20" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="26">
+      <c r="B2" s="22">
         <v>4</v>
       </c>
-      <c r="C2" s="27">
+      <c r="C2" s="23">
         <v>3</v>
       </c>
-      <c r="D2" s="27">
+      <c r="D2" s="23">
         <v>-1</v>
       </c>
-      <c r="E2" s="27">
+      <c r="E2" s="23">
         <v>0</v>
       </c>
-      <c r="F2" s="27">
+      <c r="F2" s="23">
         <v>1</v>
       </c>
-      <c r="G2" s="27">
+      <c r="G2" s="23">
         <v>2</v>
       </c>
-      <c r="H2" s="27">
+      <c r="H2" s="23">
         <v>0</v>
       </c>
-      <c r="I2" s="27">
+      <c r="I2" s="23">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="26">
+      <c r="B3" s="22">
         <v>4</v>
       </c>
-      <c r="C3" s="27">
+      <c r="C3" s="23">
         <v>-1</v>
       </c>
-      <c r="D3" s="27">
+      <c r="D3" s="23">
         <v>1</v>
       </c>
-      <c r="E3" s="27">
+      <c r="E3" s="23">
         <v>2</v>
       </c>
-      <c r="F3" s="27">
+      <c r="F3" s="23">
         <v>0</v>
       </c>
-      <c r="G3" s="27">
+      <c r="G3" s="23">
         <v>-1</v>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="23">
         <v>2</v>
       </c>
-      <c r="I3" s="27">
+      <c r="I3" s="23">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="26">
+      <c r="B4" s="22">
         <v>4</v>
       </c>
-      <c r="C4" s="27">
+      <c r="C4" s="23">
         <v>1</v>
       </c>
-      <c r="D4" s="27">
+      <c r="D4" s="23">
         <v>1</v>
       </c>
-      <c r="E4" s="27">
+      <c r="E4" s="23">
         <v>-1</v>
       </c>
-      <c r="F4" s="27">
+      <c r="F4" s="23">
         <v>2</v>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="23">
         <v>1</v>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="23">
         <v>0</v>
       </c>
-      <c r="I4" s="27">
+      <c r="I4" s="23">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="B5" s="28">
+      <c r="B5" s="24">
         <v>4</v>
       </c>
-      <c r="C5" s="27">
+      <c r="C5" s="23">
         <v>0</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="23">
         <v>2</v>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="23">
         <v>2</v>
       </c>
-      <c r="F5" s="27">
+      <c r="F5" s="23">
         <v>0</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="23">
         <v>1</v>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="23">
         <v>1</v>
       </c>
-      <c r="I5" s="27">
+      <c r="I5" s="23">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="24"/>
-      <c r="B6" s="25" t="s">
+      <c r="A6" s="20"/>
+      <c r="B6" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="25">
         <v>3</v>
       </c>
-      <c r="D6" s="29">
+      <c r="D6" s="25">
         <v>3</v>
       </c>
-      <c r="E6" s="29">
+      <c r="E6" s="25">
         <v>3</v>
       </c>
-      <c r="F6" s="29">
+      <c r="F6" s="25">
         <v>3</v>
       </c>
-      <c r="G6" s="29">
+      <c r="G6" s="25">
         <v>3</v>
       </c>
-      <c r="H6" s="29">
+      <c r="H6" s="25">
         <v>3</v>
       </c>
-      <c r="I6" s="29">
+      <c r="I6" s="25">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="24"/>
-      <c r="B7" s="34" t="s">
+      <c r="A7" s="20"/>
+      <c r="B7" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="24"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="30">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="26">
         <v>7</v>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="27">
         <v>3</v>
       </c>
-      <c r="E8" s="31">
+      <c r="E8" s="27">
         <v>4</v>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="27">
         <v>5</v>
       </c>
-      <c r="G8" s="31">
+      <c r="G8" s="27">
         <v>6</v>
       </c>
-      <c r="H8" s="31">
+      <c r="H8" s="27">
         <v>4</v>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="27">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="32">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="28">
         <v>3</v>
       </c>
-      <c r="D9" s="33">
+      <c r="D9" s="29">
         <v>5</v>
       </c>
-      <c r="E9" s="33">
+      <c r="E9" s="29">
         <v>6</v>
       </c>
-      <c r="F9" s="33">
+      <c r="F9" s="29">
         <v>4</v>
       </c>
-      <c r="G9" s="33">
+      <c r="G9" s="29">
         <v>3</v>
       </c>
-      <c r="H9" s="33">
+      <c r="H9" s="29">
         <v>6</v>
       </c>
-      <c r="I9" s="33">
+      <c r="I9" s="29">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="32">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="28">
         <v>5</v>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="29">
         <v>5</v>
       </c>
-      <c r="E10" s="33">
+      <c r="E10" s="29">
         <v>3</v>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="29">
         <v>6</v>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="29">
         <v>5</v>
       </c>
-      <c r="H10" s="33">
+      <c r="H10" s="29">
         <v>4</v>
       </c>
-      <c r="I10" s="33">
+      <c r="I10" s="29">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="24"/>
-      <c r="B11" s="24"/>
-      <c r="C11" s="32">
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="28">
         <v>4</v>
       </c>
-      <c r="D11" s="33">
+      <c r="D11" s="29">
         <v>6</v>
       </c>
-      <c r="E11" s="33">
+      <c r="E11" s="29">
         <v>6</v>
       </c>
-      <c r="F11" s="33">
+      <c r="F11" s="29">
         <v>4</v>
       </c>
-      <c r="G11" s="33">
+      <c r="G11" s="29">
         <v>5</v>
       </c>
-      <c r="H11" s="33">
+      <c r="H11" s="29">
         <v>5</v>
       </c>
-      <c r="I11" s="33">
+      <c r="I11" s="29">
         <v>4</v>
       </c>
     </row>
@@ -6394,25 +6721,25 @@
       <c r="A16" t="s">
         <v>193</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="C16" s="36" t="s">
+      <c r="C16" s="30" t="s">
         <v>197</v>
       </c>
-      <c r="D16" s="36" t="s">
+      <c r="D16" s="30" t="s">
         <v>197</v>
       </c>
-      <c r="E16" s="36" t="s">
+      <c r="E16" s="30" t="s">
         <v>198</v>
       </c>
-      <c r="F16" s="36" t="s">
+      <c r="F16" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="G16" s="36" t="s">
+      <c r="G16" s="30" t="s">
         <v>197</v>
       </c>
-      <c r="H16" s="36" t="s">
+      <c r="H16" s="30" t="s">
         <v>197</v>
       </c>
       <c r="J16" t="s">
@@ -6526,4 +6853,463 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667D7B80-3595-CB4B-B56B-C4DEC5895CBA}">
+  <dimension ref="A1:E58"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="2" customWidth="1"/>
+    <col min="4" max="4" width="1.1640625" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="32" x14ac:dyDescent="0.4">
+      <c r="A1" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+    </row>
+    <row r="2" spans="1:5" ht="24" x14ac:dyDescent="0.3">
+      <c r="A2" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37" t="s">
+        <v>207</v>
+      </c>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C4" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>213</v>
+      </c>
+      <c r="C5" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>224</v>
+      </c>
+      <c r="C6" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>223</v>
+      </c>
+      <c r="C7" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>210</v>
+      </c>
+      <c r="C8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>305</v>
+      </c>
+      <c r="C9" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>212</v>
+      </c>
+      <c r="C10" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>248</v>
+      </c>
+      <c r="C12" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>307</v>
+      </c>
+      <c r="C13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>306</v>
+      </c>
+      <c r="C14" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>244</v>
+      </c>
+      <c r="C15" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>245</v>
+      </c>
+      <c r="C16" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>242</v>
+      </c>
+      <c r="C17" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>246</v>
+      </c>
+      <c r="C18" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>243</v>
+      </c>
+      <c r="C19" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>252</v>
+      </c>
+      <c r="C20" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>253</v>
+      </c>
+      <c r="C21" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>251</v>
+      </c>
+      <c r="C22" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>254</v>
+      </c>
+      <c r="C23" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>256</v>
+      </c>
+      <c r="C24" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>255</v>
+      </c>
+      <c r="C25" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>286</v>
+      </c>
+      <c r="C26" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>284</v>
+      </c>
+      <c r="C27" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>285</v>
+      </c>
+      <c r="C28" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>308</v>
+      </c>
+      <c r="C29" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>309</v>
+      </c>
+      <c r="C30" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>302</v>
+      </c>
+      <c r="C31" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>304</v>
+      </c>
+      <c r="C32" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>265</v>
+      </c>
+      <c r="C33" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>266</v>
+      </c>
+      <c r="C34" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>261</v>
+      </c>
+      <c r="C35" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>262</v>
+      </c>
+      <c r="C36" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>263</v>
+      </c>
+      <c r="C37" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>264</v>
+      </c>
+      <c r="C38" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>267</v>
+      </c>
+      <c r="C39" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>268</v>
+      </c>
+      <c r="C40" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>270</v>
+      </c>
+      <c r="C41" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>269</v>
+      </c>
+      <c r="C42" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>209</v>
+      </c>
+      <c r="C43" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>281</v>
+      </c>
+      <c r="C44" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>283</v>
+      </c>
+      <c r="C45" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>282</v>
+      </c>
+      <c r="C46" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>303</v>
+      </c>
+      <c r="C47" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C48" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C49" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="50" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C50" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="51" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C51" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="52" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C52" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="53" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C53" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="54" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C54" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="55" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C55" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="56" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C56" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="57" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C57" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="58" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C58" t="s">
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C3:C58">
+    <sortCondition ref="C3:C58"/>
+  </sortState>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>